<commit_message>
Updated NZL model - 2025-09-22 22:37
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL/BY_Trans.xlsx
+++ b/VerveStacks_NZL/BY_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175BD090-9177-48E9-AFCC-2E73ABFECA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56CEE1D-1E6F-468E-8EF0-F70318BC75F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28702" yWindow="-98" windowWidth="28995" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="50">
   <si>
     <t>attribute</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>coal,oil</t>
+  </si>
+  <si>
+    <t>-hydro</t>
   </si>
 </sst>
 </file>
@@ -731,6 +734,9 @@
       <c r="C10" t="s">
         <v>38</v>
       </c>
+      <c r="D10" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="F10" s="3" t="s">
         <v>42</v>
       </c>

</xml_diff>